<commit_message>
feat: implement stock monitoring core logic and backfill utilities with web dashboard and historical data outputs
</commit_message>
<xml_diff>
--- a/outputs/monitor_xlsx/20260119.xlsx
+++ b/outputs/monitor_xlsx/20260119.xlsx
@@ -481,6 +481,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -823,6 +824,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -878,6 +880,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -999,7 +1002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W21"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1113,40 +1116,35 @@
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>籌碼評價</t>
+          <t>買賣券商差</t>
         </is>
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
-          <t>買賣券商差</t>
+          <t>籌碼集中度5D(%)</t>
         </is>
       </c>
       <c r="R3" s="5" t="inlineStr">
         <is>
-          <t>籌碼集中度5D(%)</t>
+          <t>借券賣出餘額</t>
         </is>
       </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
-          <t>借券賣出餘額</t>
+          <t>短回補天數</t>
         </is>
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>短回補天數</t>
+          <t>VWAP20D</t>
         </is>
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>VWAP20D</t>
+          <t>VWAP乖離(%)</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
-        <is>
-          <t>VWAP乖離(%)</t>
-        </is>
-      </c>
-      <c r="W3" s="5" t="inlineStr">
         <is>
           <t>資料來源</t>
         </is>
@@ -1204,12 +1202,7 @@
       <c r="O4" t="n">
         <v>2.41</v>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>偏空</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1247,12 +1240,7 @@
       <c r="N5" t="n">
         <v>-20235</v>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>中性</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1310,12 +1298,7 @@
       <c r="O6" t="n">
         <v>9.58</v>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>偏多</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1373,12 +1356,7 @@
       <c r="O7" t="n">
         <v>5.36</v>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>偏多</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1436,12 +1414,7 @@
       <c r="O8" t="n">
         <v>3.04</v>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>偏空</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1499,12 +1472,7 @@
       <c r="O9" t="n">
         <v>14.82</v>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>偏多</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1562,12 +1530,7 @@
       <c r="O10" t="n">
         <v>-2.59</v>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>中性</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1625,12 +1588,7 @@
       <c r="O11" t="n">
         <v>-1.43</v>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>主力積極賣出</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1688,12 +1646,7 @@
       <c r="O12" t="n">
         <v>-7.7</v>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>主力積極賣出</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1751,12 +1704,7 @@
       <c r="O13" t="n">
         <v>0</v>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>偏空</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1814,12 +1762,7 @@
       <c r="O14" t="n">
         <v>0</v>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>偏多</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1877,12 +1820,7 @@
       <c r="O15" t="n">
         <v>0</v>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>偏多</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1940,12 +1878,7 @@
       <c r="O16" t="n">
         <v>0</v>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>偏空</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2003,12 +1936,7 @@
       <c r="O17" t="n">
         <v>0</v>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>主力積極買進</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
+      <c r="V17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2063,12 +1991,7 @@
       <c r="O18" t="n">
         <v>11.98</v>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>主力積極賣出</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2126,12 +2049,7 @@
           <t>中性</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>偏多</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2189,12 +2107,7 @@
       <c r="O20" t="n">
         <v>0</v>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>偏多</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr">
+      <c r="V20" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
feat: implement stock monitor logic and generate historical market analysis reports
</commit_message>
<xml_diff>
--- a/outputs/monitor_xlsx/20260119.xlsx
+++ b/outputs/monitor_xlsx/20260119.xlsx
@@ -481,7 +481,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -824,7 +823,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -880,7 +878,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -1002,7 +999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1158,7 +1155,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0050</t>
+          <t>元大台灣50</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1166,26 +1163,26 @@
           <t>上市</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="6" t="n">
         <v>72.59999999999999</v>
       </c>
       <c r="E4" s="6" t="n">
         <v>0.83</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="6" t="n">
         <v>122970</v>
       </c>
       <c r="G4" s="6" t="n">
         <v>-32902</v>
       </c>
       <c r="H4" t="n">
-        <v>-56658</v>
+        <v>-73021</v>
       </c>
       <c r="I4" t="n">
         <v>-13557</v>
       </c>
       <c r="J4" t="n">
-        <v>8663</v>
+        <v>-6994</v>
       </c>
       <c r="K4" t="n">
         <v>26144</v>
@@ -1194,13 +1191,13 @@
         <v>7719</v>
       </c>
       <c r="M4" t="n">
-        <v>39846</v>
+        <v>38979</v>
       </c>
       <c r="N4" t="n">
         <v>-3914750</v>
       </c>
       <c r="O4" t="n">
-        <v>2.41</v>
+        <v>2.43</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -1262,26 +1259,26 @@
           <t>上市</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="7" t="n">
         <v>963</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>-0.21</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="6" t="n">
         <v>8846</v>
       </c>
       <c r="G6" s="6" t="n">
         <v>-534</v>
       </c>
       <c r="H6" t="n">
-        <v>5350</v>
+        <v>2736</v>
       </c>
       <c r="I6" t="n">
         <v>7</v>
       </c>
       <c r="J6" t="n">
-        <v>1467</v>
+        <v>1366</v>
       </c>
       <c r="K6" t="n">
         <v>234</v>
@@ -1290,13 +1287,13 @@
         <v>3222</v>
       </c>
       <c r="M6" t="n">
-        <v>17310</v>
+        <v>16878</v>
       </c>
       <c r="N6" t="n">
         <v>-78522</v>
       </c>
       <c r="O6" t="n">
-        <v>9.58</v>
+        <v>12.01</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
@@ -1320,26 +1317,26 @@
           <t>上市</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="7" t="n">
         <v>1120</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>-0.44</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="6" t="n">
         <v>12864</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>-1327</v>
       </c>
       <c r="H7" t="n">
-        <v>9030</v>
+        <v>4819</v>
       </c>
       <c r="I7" t="n">
         <v>-12</v>
       </c>
       <c r="J7" t="n">
-        <v>815</v>
+        <v>341</v>
       </c>
       <c r="K7" t="n">
         <v>425</v>
@@ -1348,13 +1345,13 @@
         <v>8803</v>
       </c>
       <c r="M7" t="n">
-        <v>38974</v>
+        <v>40133</v>
       </c>
       <c r="N7" t="n">
         <v>-648575</v>
       </c>
       <c r="O7" t="n">
-        <v>5.36</v>
+        <v>5.91</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
@@ -1378,26 +1375,26 @@
           <t>上市</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="6" t="n">
         <v>1760</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>1.15</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="6" t="n">
         <v>32242</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>-8021</v>
       </c>
       <c r="H8" t="n">
-        <v>-19427</v>
+        <v>-17193</v>
       </c>
       <c r="I8" t="n">
         <v>-1064</v>
       </c>
       <c r="J8" t="n">
-        <v>2432</v>
+        <v>1349</v>
       </c>
       <c r="K8" t="n">
         <v>2201</v>
@@ -1406,7 +1403,7 @@
         <v>20659</v>
       </c>
       <c r="M8" t="n">
-        <v>110645</v>
+        <v>108919</v>
       </c>
       <c r="N8" t="n">
         <v>-6482710</v>
@@ -1494,26 +1491,26 @@
           <t>上市</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="7" t="n">
         <v>1580</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>-2.77</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="7" t="n">
         <v>3928</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>546</v>
       </c>
       <c r="H10" t="n">
-        <v>287</v>
+        <v>458</v>
       </c>
       <c r="I10" t="n">
         <v>-417</v>
       </c>
       <c r="J10" t="n">
-        <v>-568</v>
+        <v>-910</v>
       </c>
       <c r="K10" t="n">
         <v>320</v>
@@ -1522,13 +1519,13 @@
         <v>2452</v>
       </c>
       <c r="M10" t="n">
-        <v>13738</v>
+        <v>13228</v>
       </c>
       <c r="N10" t="n">
         <v>-89502</v>
       </c>
       <c r="O10" t="n">
-        <v>-2.59</v>
+        <v>-1.25</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
@@ -1610,26 +1607,26 @@
           <t>上市</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="7" t="n">
         <v>1235</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>-1.59</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="7" t="n">
         <v>2135</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>268</v>
       </c>
       <c r="H12" t="n">
-        <v>-1183</v>
+        <v>-908</v>
       </c>
       <c r="I12" t="n">
         <v>-124</v>
       </c>
       <c r="J12" t="n">
-        <v>-123</v>
+        <v>-339</v>
       </c>
       <c r="K12" t="n">
         <v>63</v>
@@ -1638,13 +1635,13 @@
         <v>5165</v>
       </c>
       <c r="M12" t="n">
-        <v>27539</v>
+        <v>27133</v>
       </c>
       <c r="N12" t="n">
         <v>-19172</v>
       </c>
       <c r="O12" t="n">
-        <v>-7.7</v>
+        <v>-7.27</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
@@ -1658,36 +1655,28 @@
           <t>3081</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>聯亞</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>上櫃</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>1365</v>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" s="6" t="n">
+        <v>2.16</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="F13" t="n">
-        <v>9343</v>
+        <v>2182</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>-574</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>-574</v>
       </c>
       <c r="H13" t="n">
-        <v>-1193</v>
+        <v>-1603</v>
       </c>
       <c r="I13" t="n">
         <v>230</v>
       </c>
       <c r="J13" t="n">
-        <v>280</v>
+        <v>444</v>
       </c>
       <c r="K13" t="n">
         <v>9</v>
@@ -1696,7 +1685,7 @@
         <v>31</v>
       </c>
       <c r="M13" t="n">
-        <v>902</v>
+        <v>570</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -1832,36 +1821,28 @@
           <t>4979</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>華星光</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>上櫃</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>400</v>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" s="6" t="n">
+        <v>9.94</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>-4.42</v>
-      </c>
-      <c r="F16" t="n">
-        <v>7565</v>
+        <v>32773</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>2080</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>2080</v>
       </c>
       <c r="H16" t="n">
-        <v>-3592</v>
+        <v>341</v>
       </c>
       <c r="I16" t="n">
         <v>-1256</v>
       </c>
       <c r="J16" t="n">
-        <v>-2892</v>
+        <v>-3758</v>
       </c>
       <c r="K16" t="n">
         <v>-113</v>
@@ -1870,7 +1851,7 @@
         <v>-1182</v>
       </c>
       <c r="M16" t="n">
-        <v>-2181</v>
+        <v>-3103</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
@@ -2008,46 +1989,46 @@
           <t>智邦</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
         <v>1165</v>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="E19" s="7" t="n">
         <v>-5.28</v>
       </c>
-      <c r="E19" s="7" t="n">
+      <c r="F19" s="6" t="n">
         <v>4631</v>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="G19" s="6" t="n">
         <v>-160</v>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="H19" t="n">
         <v>198</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>-514</v>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>-293</v>
       </c>
-      <c r="J19" t="n">
+      <c r="K19" t="n">
         <v>251</v>
       </c>
-      <c r="K19" t="n">
+      <c r="L19" t="n">
         <v>2643</v>
       </c>
-      <c r="L19" t="n">
+      <c r="M19" t="n">
         <v>13885</v>
       </c>
-      <c r="M19" t="n">
+      <c r="N19" t="n">
         <v>-140153</v>
       </c>
-      <c r="N19" t="n">
-        <v>-3.39</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>中性</t>
-        </is>
+      <c r="O19" t="n">
+        <v>-4.07</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
@@ -2164,6 +2145,249 @@
         <is>
           <t>偏多</t>
         </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2360</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>致茂</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>950</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>-3.94</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>2893</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>392</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1342</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-347</v>
+      </c>
+      <c r="J22" t="n">
+        <v>-835</v>
+      </c>
+      <c r="K22" t="n">
+        <v>140</v>
+      </c>
+      <c r="L22" t="n">
+        <v>907</v>
+      </c>
+      <c r="M22" t="n">
+        <v>4860</v>
+      </c>
+      <c r="N22" t="n">
+        <v>-106274</v>
+      </c>
+      <c r="O22" t="n">
+        <v>-1.04</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>6515</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>穎崴</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>3460</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>-2.12</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>487</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>-46</v>
+      </c>
+      <c r="H23" t="n">
+        <v>68</v>
+      </c>
+      <c r="I23" t="n">
+        <v>-30</v>
+      </c>
+      <c r="J23" t="n">
+        <v>32</v>
+      </c>
+      <c r="K23" t="n">
+        <v>12</v>
+      </c>
+      <c r="L23" t="n">
+        <v>465</v>
+      </c>
+      <c r="M23" t="n">
+        <v>2511</v>
+      </c>
+      <c r="N23" t="n">
+        <v>-8855</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>6187</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" s="7" t="n">
+        <v>-2.64</v>
+      </c>
+      <c r="E24" t="n">
+        <v>6341</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>-32</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>-32</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-663</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>-369</v>
+      </c>
+      <c r="K24" t="n">
+        <v>-10</v>
+      </c>
+      <c r="L24" t="n">
+        <v>-17</v>
+      </c>
+      <c r="M24" t="n">
+        <v>163</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>6640</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" s="7" t="n">
+        <v>-6.07</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1168</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="H25" t="n">
+        <v>45</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>-10</v>
+      </c>
+      <c r="K25" t="n">
+        <v>18</v>
+      </c>
+      <c r="L25" t="n">
+        <v>-189</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-193</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>3167</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>大量</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>-2.44</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>6438</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>-728</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-1104</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-472</v>
+      </c>
+      <c r="J26" t="n">
+        <v>-1248</v>
+      </c>
+      <c r="K26" t="n">
+        <v>81</v>
+      </c>
+      <c r="L26" t="n">
+        <v>6780</v>
+      </c>
+      <c r="M26" t="n">
+        <v>33289</v>
+      </c>
+      <c r="N26" t="n">
+        <v>-21445</v>
+      </c>
+      <c r="O26" t="n">
+        <v>-2.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>